<commit_message>
New monster: red crab (ปูแดง Lv.3)
- Balance sheet: new row 43 (mob039) on มอน, HP x1.3 / EXP x1.15 -> HP 81, DEF 1, ATK 10, EXP 43; JSON re-exported
- art/monsters/red-crab: source, 4x4 sheet (walk/attack/hit/death, 35x28) and 6-frame idle (35x33)
- 6 spawn on the first map, fight back like the mud crab, no drop yet (waiting for an item image)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/balance/siam-legends-balance.xlsx
+++ b/balance/siam-legends-balance.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kenio\Downloads\siam-legends-online (2)\siam-legends-online\balance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F6CFE75-7857-4E65-8AD0-513E1E8B4F7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4D56A65-6C81-4F9B-8778-C8DB7F9A73D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -117,7 +117,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="203">
   <si>
     <t>Siam Legends Online — ตารางสมดุลเกม (มอน / เลเวล / EXP)</t>
   </si>
@@ -723,6 +723,9 @@
   </si>
   <si>
     <t>บอสสุดท้าย</t>
+  </si>
+  <si>
+    <t>ปูแดง</t>
   </si>
 </sst>
 </file>
@@ -9844,7 +9847,7 @@
         <v>68</v>
       </c>
       <c r="G101" s="26">
-        <f t="shared" ref="G101:G132" si="21">MAX(1,D101-F101)</f>
+        <f t="shared" ref="G101:G104" si="21">MAX(1,D101-F101)</f>
         <v>1297.4000000000001</v>
       </c>
       <c r="H101" s="25">
@@ -9864,11 +9867,11 @@
         <v>686.62742622201927</v>
       </c>
       <c r="L101" s="25">
-        <f t="shared" ref="L101:L132" si="22">K101*60/J101</f>
+        <f t="shared" ref="L101:L104" si="22">K101*60/J101</f>
         <v>6058.4772901942879</v>
       </c>
       <c r="M101" s="25">
-        <f t="shared" ref="M101:M132" si="23">MAX(1,ROUND(B101/L101,0))</f>
+        <f t="shared" ref="M101:M104" si="23">MAX(1,ROUND(B101/L101,0))</f>
         <v>2260</v>
       </c>
       <c r="N101" s="25">
@@ -9884,7 +9887,7 @@
         <v>6058</v>
       </c>
       <c r="Q101" s="27">
-        <f t="shared" ref="Q101:Q132" si="24">P101*J101/60</f>
+        <f t="shared" ref="Q101:Q104" si="24">P101*J101/60</f>
         <v>686.57333333333338</v>
       </c>
       <c r="R101" s="26">
@@ -10120,7 +10123,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:O42"/>
+  <dimension ref="A1:O43"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -12243,6 +12246,53 @@
         <v>201</v>
       </c>
     </row>
+    <row r="43" spans="1:15">
+      <c r="A43" s="30" t="s">
+        <v>202</v>
+      </c>
+      <c r="B43" s="31" t="s">
+        <v>118</v>
+      </c>
+      <c r="C43" s="31">
+        <v>3</v>
+      </c>
+      <c r="D43" s="31" t="s">
+        <v>119</v>
+      </c>
+      <c r="E43" s="31" t="s">
+        <v>120</v>
+      </c>
+      <c r="F43" s="29">
+        <v>1.3</v>
+      </c>
+      <c r="G43" s="29">
+        <v>1.1499999999999999</v>
+      </c>
+      <c r="H43" s="25">
+        <f>ROUND(INDEX(เลเวล!$H$5:$H$104,C43)*F43*IF(D43="บอส",ตั้งค่า!$C$29,1),0)</f>
+        <v>81</v>
+      </c>
+      <c r="I43" s="25">
+        <f>ROUND(INDEX(เลเวล!$F$5:$F$104,C43)*IF(D43="บอส",ตั้งค่า!$C$32,1),0)</f>
+        <v>1</v>
+      </c>
+      <c r="J43" s="25">
+        <f>ROUND(INDEX(เลเวล!$I$5:$I$104,C43)*IF(D43="บอส",ตั้งค่า!$C$31,1),0)</f>
+        <v>10</v>
+      </c>
+      <c r="K43" s="25">
+        <f>ROUND(INDEX(เลเวล!$M$5:$M$104,C43)*G43*IF(D43="บอส",ตั้งค่า!$C$30,1),0)</f>
+        <v>43</v>
+      </c>
+      <c r="L43" s="25">
+        <f>ROUND(INDEX(เลเวล!$N$5:$N$104,C43)*IF(D43="บอส",ตั้งค่า!$C$33,1),0)</f>
+        <v>15</v>
+      </c>
+      <c r="M43" s="25">
+        <f>ROUND(INDEX(เลเวล!$O$5:$O$104,C43)*IF(D43="บอส",ตั้งค่า!$C$33,1),0)</f>
+        <v>22</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Add scarecrow and lotus frog to the map; grasshopper/octopus art ready; monk sliced
- Sliced with slice_sheet.py (5 poses each): scarecrow, lotus frog, grasshopper, octopus (hit/death/idle
  as separate sheets), monk NPC idle
- Scarecrow = mob007 Lv8 in the paddies, drops straw hat; lotus frog = mob005 Lv5 (renamed from กบเขียว
  in the balance sheet) around a new lotus pond in the residential area, drops lotus
- Grasshopper (sickle) and octopus (iron helmet): art + items ready, count 0 (no level yet)
- New items with 64/32/16 icons; sai_sin (no image) shows its name in the bag
- tools/fix_checker.py, tools/regrid_sheet.py; shared/data/npcs.json, quests.json (quest system pending)
- CLAUDE.md: monster/NPC status table, new tools, quest-giver rule, how to hand in new art

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/balance/siam-legends-balance.xlsx
+++ b/balance/siam-legends-balance.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kenio\Downloads\siam-legends-online (2)\siam-legends-online\balance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4D56A65-6C81-4F9B-8778-C8DB7F9A73D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{374DD698-A2AD-4EEE-B88D-F7C5F97BBC14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -503,9 +503,6 @@
     <t>ช้าแต่ถึก</t>
   </si>
   <si>
-    <t>กบเขียว</t>
-  </si>
-  <si>
     <t>กระโดดไกล</t>
   </si>
   <si>
@@ -726,6 +723,9 @@
   </si>
   <si>
     <t>ปูแดง</t>
+  </si>
+  <si>
+    <t>กบบัว</t>
   </si>
 </sst>
 </file>
@@ -10414,7 +10414,7 @@
     </row>
     <row r="9" spans="1:15">
       <c r="A9" s="3" t="s">
-        <v>128</v>
+        <v>202</v>
       </c>
       <c r="B9" s="28" t="s">
         <v>118</v>
@@ -10463,12 +10463,12 @@
         <v>4</v>
       </c>
       <c r="O9" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="10" spans="1:15">
       <c r="A10" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B10" s="28" t="s">
         <v>118</v>
@@ -10480,7 +10480,7 @@
         <v>119</v>
       </c>
       <c r="E10" s="28" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F10" s="29">
         <v>1.2</v>
@@ -10517,12 +10517,12 @@
         <v>5</v>
       </c>
       <c r="O10" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="11" spans="1:15">
       <c r="A11" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B11" s="28" t="s">
         <v>118</v>
@@ -10534,7 +10534,7 @@
         <v>119</v>
       </c>
       <c r="E11" s="28" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F11" s="29">
         <v>1</v>
@@ -10571,12 +10571,12 @@
         <v>5</v>
       </c>
       <c r="O11" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="12" spans="1:15">
       <c r="A12" s="30" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B12" s="31" t="s">
         <v>118</v>
@@ -10585,10 +10585,10 @@
         <v>10</v>
       </c>
       <c r="D12" s="31" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E12" s="31" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F12" s="29">
         <v>1</v>
@@ -10625,15 +10625,15 @@
         <v>161</v>
       </c>
       <c r="O12" s="3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="13" spans="1:15">
       <c r="A13" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="B13" s="28" t="s">
         <v>138</v>
-      </c>
-      <c r="B13" s="28" t="s">
-        <v>139</v>
       </c>
       <c r="C13" s="28">
         <v>11</v>
@@ -10679,15 +10679,15 @@
         <v>4</v>
       </c>
       <c r="O13" s="3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="14" spans="1:15">
       <c r="A14" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B14" s="28" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C14" s="28">
         <v>13</v>
@@ -10696,7 +10696,7 @@
         <v>119</v>
       </c>
       <c r="E14" s="28" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F14" s="29">
         <v>1</v>
@@ -10733,15 +10733,15 @@
         <v>5</v>
       </c>
       <c r="O14" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="15" spans="1:15">
       <c r="A15" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B15" s="28" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C15" s="28">
         <v>14</v>
@@ -10787,15 +10787,15 @@
         <v>5</v>
       </c>
       <c r="O15" s="3" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="16" spans="1:15">
       <c r="A16" s="3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B16" s="28" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C16" s="28">
         <v>16</v>
@@ -10804,7 +10804,7 @@
         <v>119</v>
       </c>
       <c r="E16" s="28" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F16" s="29">
         <v>0.9</v>
@@ -10841,15 +10841,15 @@
         <v>4</v>
       </c>
       <c r="O16" s="3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="17" spans="1:15">
       <c r="A17" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B17" s="28" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C17" s="28">
         <v>18</v>
@@ -10858,7 +10858,7 @@
         <v>119</v>
       </c>
       <c r="E17" s="28" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F17" s="29">
         <v>1.4</v>
@@ -10895,24 +10895,24 @@
         <v>6</v>
       </c>
       <c r="O17" s="3" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="18" spans="1:15">
       <c r="A18" s="30" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B18" s="31" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C18" s="31">
         <v>20</v>
       </c>
       <c r="D18" s="31" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E18" s="31" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F18" s="29">
         <v>1</v>
@@ -10949,15 +10949,15 @@
         <v>160</v>
       </c>
       <c r="O18" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="19" spans="1:15">
       <c r="A19" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="B19" s="28" t="s">
         <v>151</v>
-      </c>
-      <c r="B19" s="28" t="s">
-        <v>152</v>
       </c>
       <c r="C19" s="28">
         <v>22</v>
@@ -10966,7 +10966,7 @@
         <v>119</v>
       </c>
       <c r="E19" s="28" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F19" s="29">
         <v>1.2</v>
@@ -11003,15 +11003,15 @@
         <v>5</v>
       </c>
       <c r="O19" s="3" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="20" spans="1:15">
       <c r="A20" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B20" s="28" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C20" s="28">
         <v>24</v>
@@ -11020,7 +11020,7 @@
         <v>119</v>
       </c>
       <c r="E20" s="28" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F20" s="29">
         <v>0.8</v>
@@ -11057,15 +11057,15 @@
         <v>4</v>
       </c>
       <c r="O20" s="3" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="21" spans="1:15">
       <c r="A21" s="3" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B21" s="28" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C21" s="28">
         <v>26</v>
@@ -11074,7 +11074,7 @@
         <v>119</v>
       </c>
       <c r="E21" s="28" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F21" s="29">
         <v>0.9</v>
@@ -11111,15 +11111,15 @@
         <v>4</v>
       </c>
       <c r="O21" s="3" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="22" spans="1:15">
       <c r="A22" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B22" s="28" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C22" s="28">
         <v>29</v>
@@ -11128,7 +11128,7 @@
         <v>119</v>
       </c>
       <c r="E22" s="28" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F22" s="29">
         <v>1.1000000000000001</v>
@@ -11165,15 +11165,15 @@
         <v>5</v>
       </c>
       <c r="O22" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="23" spans="1:15">
       <c r="A23" s="3" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B23" s="28" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C23" s="28">
         <v>32</v>
@@ -11182,7 +11182,7 @@
         <v>119</v>
       </c>
       <c r="E23" s="28" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F23" s="29">
         <v>1.6</v>
@@ -11219,24 +11219,24 @@
         <v>7</v>
       </c>
       <c r="O23" s="3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="24" spans="1:15">
       <c r="A24" s="30" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B24" s="31" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C24" s="31">
         <v>35</v>
       </c>
       <c r="D24" s="31" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E24" s="31" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F24" s="29">
         <v>1</v>
@@ -11273,15 +11273,15 @@
         <v>161</v>
       </c>
       <c r="O24" s="3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="25" spans="1:15">
       <c r="A25" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="B25" s="28" t="s">
         <v>164</v>
-      </c>
-      <c r="B25" s="28" t="s">
-        <v>165</v>
       </c>
       <c r="C25" s="28">
         <v>38</v>
@@ -11290,7 +11290,7 @@
         <v>119</v>
       </c>
       <c r="E25" s="28" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F25" s="29">
         <v>1</v>
@@ -11327,15 +11327,15 @@
         <v>5</v>
       </c>
       <c r="O25" s="3" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="26" spans="1:15">
       <c r="A26" s="3" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B26" s="28" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C26" s="28">
         <v>41</v>
@@ -11344,7 +11344,7 @@
         <v>119</v>
       </c>
       <c r="E26" s="28" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F26" s="29">
         <v>0.8</v>
@@ -11381,15 +11381,15 @@
         <v>4</v>
       </c>
       <c r="O26" s="3" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="27" spans="1:15">
       <c r="A27" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B27" s="28" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C27" s="28">
         <v>43</v>
@@ -11398,7 +11398,7 @@
         <v>119</v>
       </c>
       <c r="E27" s="28" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F27" s="29">
         <v>1</v>
@@ -11435,15 +11435,15 @@
         <v>4</v>
       </c>
       <c r="O27" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="28" spans="1:15">
       <c r="A28" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B28" s="28" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C28" s="28">
         <v>46</v>
@@ -11452,7 +11452,7 @@
         <v>119</v>
       </c>
       <c r="E28" s="28" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F28" s="29">
         <v>1.2</v>
@@ -11489,15 +11489,15 @@
         <v>5</v>
       </c>
       <c r="O28" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="29" spans="1:15">
       <c r="A29" s="3" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B29" s="28" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C29" s="28">
         <v>50</v>
@@ -11506,7 +11506,7 @@
         <v>119</v>
       </c>
       <c r="E29" s="28" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F29" s="29">
         <v>1.5</v>
@@ -11543,24 +11543,24 @@
         <v>7</v>
       </c>
       <c r="O29" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="30" spans="1:15">
       <c r="A30" s="30" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B30" s="31" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C30" s="31">
         <v>55</v>
       </c>
       <c r="D30" s="31" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E30" s="31" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F30" s="29">
         <v>1</v>
@@ -11597,15 +11597,15 @@
         <v>160</v>
       </c>
       <c r="O30" s="3" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="31" spans="1:15">
       <c r="A31" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="B31" s="28" t="s">
         <v>177</v>
-      </c>
-      <c r="B31" s="28" t="s">
-        <v>178</v>
       </c>
       <c r="C31" s="28">
         <v>58</v>
@@ -11614,7 +11614,7 @@
         <v>119</v>
       </c>
       <c r="E31" s="28" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F31" s="29">
         <v>1.3</v>
@@ -11651,15 +11651,15 @@
         <v>6</v>
       </c>
       <c r="O31" s="3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="32" spans="1:15">
       <c r="A32" s="3" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B32" s="28" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C32" s="28">
         <v>61</v>
@@ -11668,7 +11668,7 @@
         <v>119</v>
       </c>
       <c r="E32" s="28" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F32" s="29">
         <v>1.2</v>
@@ -11705,15 +11705,15 @@
         <v>5</v>
       </c>
       <c r="O32" s="3" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="33" spans="1:15">
       <c r="A33" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B33" s="28" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C33" s="28">
         <v>64</v>
@@ -11722,7 +11722,7 @@
         <v>119</v>
       </c>
       <c r="E33" s="28" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F33" s="29">
         <v>0.9</v>
@@ -11759,15 +11759,15 @@
         <v>4</v>
       </c>
       <c r="O33" s="3" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="34" spans="1:15">
       <c r="A34" s="3" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B34" s="28" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C34" s="28">
         <v>67</v>
@@ -11776,7 +11776,7 @@
         <v>119</v>
       </c>
       <c r="E34" s="28" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F34" s="29">
         <v>1.5</v>
@@ -11813,15 +11813,15 @@
         <v>6</v>
       </c>
       <c r="O34" s="3" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="35" spans="1:15">
       <c r="A35" s="3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B35" s="28" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C35" s="28">
         <v>71</v>
@@ -11830,7 +11830,7 @@
         <v>119</v>
       </c>
       <c r="E35" s="28" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F35" s="29">
         <v>1.2</v>
@@ -11867,24 +11867,24 @@
         <v>5</v>
       </c>
       <c r="O35" s="3" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="36" spans="1:15">
       <c r="A36" s="30" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B36" s="31" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C36" s="31">
         <v>75</v>
       </c>
       <c r="D36" s="31" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E36" s="31" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F36" s="29">
         <v>1</v>
@@ -11921,15 +11921,15 @@
         <v>161</v>
       </c>
       <c r="O36" s="3" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="37" spans="1:15">
       <c r="A37" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="B37" s="28" t="s">
         <v>190</v>
-      </c>
-      <c r="B37" s="28" t="s">
-        <v>191</v>
       </c>
       <c r="C37" s="28">
         <v>80</v>
@@ -11938,7 +11938,7 @@
         <v>119</v>
       </c>
       <c r="E37" s="28" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F37" s="29">
         <v>1.2</v>
@@ -11975,15 +11975,15 @@
         <v>5</v>
       </c>
       <c r="O37" s="3" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="38" spans="1:15">
       <c r="A38" s="3" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B38" s="28" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C38" s="28">
         <v>84</v>
@@ -11992,7 +11992,7 @@
         <v>119</v>
       </c>
       <c r="E38" s="28" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F38" s="29">
         <v>1.1000000000000001</v>
@@ -12029,15 +12029,15 @@
         <v>5</v>
       </c>
       <c r="O38" s="3" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="39" spans="1:15">
       <c r="A39" s="3" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B39" s="28" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C39" s="28">
         <v>88</v>
@@ -12046,7 +12046,7 @@
         <v>119</v>
       </c>
       <c r="E39" s="28" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F39" s="29">
         <v>0.9</v>
@@ -12083,15 +12083,15 @@
         <v>4</v>
       </c>
       <c r="O39" s="3" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="40" spans="1:15">
       <c r="A40" s="3" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B40" s="28" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C40" s="28">
         <v>92</v>
@@ -12100,7 +12100,7 @@
         <v>119</v>
       </c>
       <c r="E40" s="28" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F40" s="29">
         <v>1</v>
@@ -12137,15 +12137,15 @@
         <v>4</v>
       </c>
       <c r="O40" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="41" spans="1:15">
       <c r="A41" s="3" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B41" s="28" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C41" s="28">
         <v>96</v>
@@ -12154,7 +12154,7 @@
         <v>119</v>
       </c>
       <c r="E41" s="28" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F41" s="29">
         <v>1.3</v>
@@ -12194,19 +12194,19 @@
     </row>
     <row r="42" spans="1:15">
       <c r="A42" s="30" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B42" s="31" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C42" s="31">
         <v>100</v>
       </c>
       <c r="D42" s="31" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E42" s="31" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F42" s="29">
         <v>1</v>
@@ -12243,12 +12243,12 @@
         <v>160</v>
       </c>
       <c r="O42" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="43" spans="1:15">
       <c r="A43" s="30" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B43" s="31" t="s">
         <v>118</v>

</xml_diff>

<commit_message>
Map from the user's layout JSON; grasshopper Lv10 and octopus Lv12 spawn
- shared/data/maps/ban-pak-ao.json (60x44): terrain, props at pixel anchors, start, NPC spots, spawn boxes
- shared/map.ts reads the layout instead of hand-placed code; name aliases for props and monsters,
  footprint widths for big props, gate blocks only its posts, pier walkable over water
- Monster counts/zones come from the layout spawns: mud crab 10, red crab 8, lotus frog 6,
  scarecrow 4, grasshopper 5, octopus 5
- Balance sheet: appended ตั๊กแตนเคียว Lv10 (mob040) and หมึกหมวกเหล็ก Lv12 (mob041); JSON re-exported
- Migration 0006 moves characters to the new start (29,5)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/balance/siam-legends-balance.xlsx
+++ b/balance/siam-legends-balance.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kenio\Downloads\siam-legends-online (2)\siam-legends-online\balance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{374DD698-A2AD-4EEE-B88D-F7C5F97BBC14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5987B0D-99F5-40F8-ADCF-115C9207F7B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -117,7 +117,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="206">
   <si>
     <t>Siam Legends Online — ตารางสมดุลเกม (มอน / เลเวล / EXP)</t>
   </si>
@@ -726,6 +726,15 @@
   </si>
   <si>
     <t>กบบัว</t>
+  </si>
+  <si>
+    <t>ตั๊กแตนเคียว</t>
+  </si>
+  <si>
+    <t>บ้านปากอ่าว</t>
+  </si>
+  <si>
+    <t>หมึกหมวกเหล็ก</t>
   </si>
 </sst>
 </file>
@@ -10123,7 +10132,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:O43"/>
+  <dimension ref="A1:O45"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -12293,6 +12302,100 @@
         <v>22</v>
       </c>
     </row>
+    <row r="44" spans="1:15">
+      <c r="A44" s="30" t="s">
+        <v>203</v>
+      </c>
+      <c r="B44" s="31" t="s">
+        <v>204</v>
+      </c>
+      <c r="C44" s="31">
+        <v>10</v>
+      </c>
+      <c r="D44" s="31" t="s">
+        <v>119</v>
+      </c>
+      <c r="E44" s="31" t="s">
+        <v>120</v>
+      </c>
+      <c r="F44" s="29">
+        <v>1</v>
+      </c>
+      <c r="G44" s="29">
+        <v>1</v>
+      </c>
+      <c r="H44" s="25">
+        <f>ROUND(INDEX(เลเวล!$H$5:$H$104,C44)*F44*IF(D44="บอส",ตั้งค่า!$C$29,1),0)</f>
+        <v>136</v>
+      </c>
+      <c r="I44" s="25">
+        <f>ROUND(INDEX(เลเวล!$F$5:$F$104,C44)*IF(D44="บอส",ตั้งค่า!$C$32,1),0)</f>
+        <v>2</v>
+      </c>
+      <c r="J44" s="25">
+        <f>ROUND(INDEX(เลเวล!$I$5:$I$104,C44)*IF(D44="บอส",ตั้งค่า!$C$31,1),0)</f>
+        <v>18</v>
+      </c>
+      <c r="K44" s="25">
+        <f>ROUND(INDEX(เลเวล!$M$5:$M$104,C44)*G44*IF(D44="บอส",ตั้งค่า!$C$30,1),0)</f>
+        <v>215</v>
+      </c>
+      <c r="L44" s="25">
+        <f>ROUND(INDEX(เลเวล!$N$5:$N$104,C44)*IF(D44="บอส",ตั้งค่า!$C$33,1),0)</f>
+        <v>86</v>
+      </c>
+      <c r="M44" s="25">
+        <f>ROUND(INDEX(เลเวล!$O$5:$O$104,C44)*IF(D44="บอส",ตั้งค่า!$C$33,1),0)</f>
+        <v>129</v>
+      </c>
+    </row>
+    <row r="45" spans="1:15">
+      <c r="A45" s="30" t="s">
+        <v>205</v>
+      </c>
+      <c r="B45" s="31" t="s">
+        <v>204</v>
+      </c>
+      <c r="C45" s="31">
+        <v>12</v>
+      </c>
+      <c r="D45" s="31" t="s">
+        <v>119</v>
+      </c>
+      <c r="E45" s="31" t="s">
+        <v>120</v>
+      </c>
+      <c r="F45" s="29">
+        <v>1</v>
+      </c>
+      <c r="G45" s="29">
+        <v>1</v>
+      </c>
+      <c r="H45" s="25">
+        <f>ROUND(INDEX(เลเวล!$H$5:$H$104,C45)*F45*IF(D45="บอส",ตั้งค่า!$C$29,1),0)</f>
+        <v>161</v>
+      </c>
+      <c r="I45" s="25">
+        <f>ROUND(INDEX(เลเวล!$F$5:$F$104,C45)*IF(D45="บอส",ตั้งค่า!$C$32,1),0)</f>
+        <v>2</v>
+      </c>
+      <c r="J45" s="25">
+        <f>ROUND(INDEX(เลเวล!$I$5:$I$104,C45)*IF(D45="บอส",ตั้งค่า!$C$31,1),0)</f>
+        <v>21</v>
+      </c>
+      <c r="K45" s="25">
+        <f>ROUND(INDEX(เลเวล!$M$5:$M$104,C45)*G45*IF(D45="บอส",ตั้งค่า!$C$30,1),0)</f>
+        <v>265</v>
+      </c>
+      <c r="L45" s="25">
+        <f>ROUND(INDEX(เลเวล!$N$5:$N$104,C45)*IF(D45="บอส",ตั้งค่า!$C$33,1),0)</f>
+        <v>106</v>
+      </c>
+      <c r="M45" s="25">
+        <f>ROUND(INDEX(เลเวล!$O$5:$O$104,C45)*IF(D45="บอส",ตั้งค่า!$C$33,1),0)</f>
+        <v>159</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>